<commit_message>
mejoras en migraciones historial y mas cosas
</commit_message>
<xml_diff>
--- a/docs/Exels/NOMENCLATURA RUTH.xlsx
+++ b/docs/Exels/NOMENCLATURA RUTH.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VENTAS-02\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andres\Documents\GitHub\SAM_Construcciones\docs\Exels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="186" documentId="13_ncr:1_{96400108-F293-4404-BEA5-4BEC1E51A280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DA31FE0-32A1-4DC1-BEFD-46874F1B9830}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38C110E-B3B8-40B9-88EB-0B61B423DB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{54E3828D-035F-40CD-B6FC-BEDE3347E965}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{54E3828D-035F-40CD-B6FC-BEDE3347E965}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -27,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,23 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
-  <si>
-    <t>EDIFICIO RUTH ESTHER</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="32">
   <si>
     <t>ESTATUS</t>
   </si>
   <si>
-    <t>NIVEL</t>
-  </si>
-  <si>
-    <t>NÚMERO</t>
-  </si>
-  <si>
-    <t>ADQUIRIENTE (S)</t>
-  </si>
-  <si>
     <t>CARACTERISTICAS</t>
   </si>
   <si>
@@ -62,12 +50,6 @@
     <t>INMOBILIARIA</t>
   </si>
   <si>
-    <t>PRECIOS EN RD</t>
-  </si>
-  <si>
-    <t>INICIAL 20%</t>
-  </si>
-  <si>
     <t>SEPARACIÓN</t>
   </si>
   <si>
@@ -135,6 +117,21 @@
   </si>
   <si>
     <t>3 HABITACIONES, SALA, COMEDOR, COCINA, 2 BAÑOS, CLOSET,WALKING CLOSET, AREA DE LAVADO, MAS 142.9 M DE TERRAZA DESTECHADA Y 2 PARQUEOS</t>
+  </si>
+  <si>
+    <t>PISO</t>
+  </si>
+  <si>
+    <t>unidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INICIAL </t>
+  </si>
+  <si>
+    <t>PRECIO</t>
+  </si>
+  <si>
+    <t>cliente</t>
   </si>
 </sst>
 </file>
@@ -147,7 +144,7 @@
     <numFmt numFmtId="164" formatCode="[$$-1C0A]#,##0.00_);\([$$-1C0A]#,##0.00\)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,9 +345,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -358,9 +353,12 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <font>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -375,12 +373,9 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -718,25 +713,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M16"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="4" max="4" width="27.28515625" customWidth="1"/>
-    <col min="5" max="5" width="64.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.125" customWidth="1"/>
+    <col min="4" max="4" width="27.25" customWidth="1"/>
+    <col min="5" max="5" width="64.75" customWidth="1"/>
+    <col min="6" max="6" width="13.375" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
+    <col min="9" max="9" width="18.875" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="24.28515625" customWidth="1"/>
-    <col min="12" max="12" width="24.85546875" customWidth="1"/>
-    <col min="13" max="13" width="26.28515625" customWidth="1"/>
+    <col min="11" max="11" width="24.25" customWidth="1"/>
+    <col min="12" max="12" width="24.875" customWidth="1"/>
+    <col min="13" max="13" width="26.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27">
-      <c r="B1" s="15" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.35">
+      <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
@@ -749,50 +742,50 @@
       <c r="L1" s="15"/>
       <c r="M1" s="15"/>
     </row>
-    <row r="2" spans="1:13" ht="40.5" customHeight="1">
+    <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="H2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:13" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="47.25" customHeight="1">
-      <c r="A3" s="12" t="s">
-        <v>14</v>
       </c>
       <c r="B3" s="13">
         <v>2</v>
@@ -801,16 +794,16 @@
         <v>201</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F3" s="3">
         <v>119</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H3" s="8">
         <f>9600000-480000</f>
@@ -837,9 +830,9 @@
         <v>7296000</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="50.25" customHeight="1">
+    <row r="4" spans="1:13" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B4" s="13">
         <v>2</v>
@@ -848,16 +841,16 @@
         <v>202</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F4" s="3">
         <v>110.5</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H4" s="8">
         <v>7950000</v>
@@ -883,9 +876,9 @@
         <v>6360000</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="61.5" customHeight="1">
+    <row r="5" spans="1:13" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B5" s="13">
         <v>2</v>
@@ -894,16 +887,16 @@
         <v>203</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F5" s="3">
         <v>138</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H5" s="8">
         <f>8950000-447500</f>
@@ -922,7 +915,7 @@
         <v>1275375</v>
       </c>
       <c r="L5" s="6">
-        <f t="shared" ref="L4:L14" si="4">+K5/13</f>
+        <f t="shared" ref="L5" si="4">+K5/13</f>
         <v>98105.769230769234</v>
       </c>
       <c r="M5" s="9">
@@ -930,9 +923,9 @@
         <v>6802000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="37.5" customHeight="1">
+    <row r="6" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B6" s="13">
         <v>3</v>
@@ -941,16 +934,16 @@
         <v>301</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F6" s="3">
         <v>119</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H6" s="10">
         <f>8600000-430000</f>
@@ -969,7 +962,7 @@
         <v>1225500</v>
       </c>
       <c r="L6" s="6">
-        <f>+K6/12</f>
+        <f t="shared" ref="L6:L14" si="5">+K6/12</f>
         <v>102125</v>
       </c>
       <c r="M6" s="9">
@@ -977,9 +970,9 @@
         <v>6536000</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="37.5" customHeight="1">
+    <row r="7" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B7" s="13">
         <v>3</v>
@@ -988,10 +981,10 @@
         <v>302</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F7" s="3">
         <v>110.5</v>
@@ -1014,7 +1007,7 @@
         <v>1192500</v>
       </c>
       <c r="L7" s="6">
-        <f>+K7/12</f>
+        <f t="shared" si="5"/>
         <v>99375</v>
       </c>
       <c r="M7" s="9">
@@ -1022,9 +1015,9 @@
         <v>6360000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="36" customHeight="1">
+    <row r="8" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B8" s="13">
         <v>3</v>
@@ -1033,16 +1026,16 @@
         <v>303</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F8" s="3">
         <v>138</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H8" s="10">
         <v>9050000</v>
@@ -1060,7 +1053,7 @@
         <v>1357500</v>
       </c>
       <c r="L8" s="6">
-        <f>+K8/12</f>
+        <f t="shared" si="5"/>
         <v>113125</v>
       </c>
       <c r="M8" s="9">
@@ -1068,9 +1061,9 @@
         <v>7240000</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="30">
+    <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B9" s="13">
         <v>4</v>
@@ -1079,16 +1072,16 @@
         <v>401</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F9" s="3">
         <v>119</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H9" s="8">
         <f>H6+200000</f>
@@ -1107,7 +1100,7 @@
         <v>1255500</v>
       </c>
       <c r="L9" s="6">
-        <f>+K9/12</f>
+        <f t="shared" si="5"/>
         <v>104625</v>
       </c>
       <c r="M9" s="9">
@@ -1115,9 +1108,9 @@
         <v>6696000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="30">
+    <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B10" s="13">
         <v>4</v>
@@ -1126,16 +1119,16 @@
         <v>402</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F10" s="3">
         <v>110.5</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H10" s="8">
         <v>7500000</v>
@@ -1153,7 +1146,7 @@
         <v>1125000</v>
       </c>
       <c r="L10" s="6">
-        <f>+K10/12</f>
+        <f t="shared" si="5"/>
         <v>93750</v>
       </c>
       <c r="M10" s="9">
@@ -1161,9 +1154,9 @@
         <v>6000000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="34.5" customHeight="1">
+    <row r="11" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B11" s="13">
         <v>4</v>
@@ -1172,16 +1165,16 @@
         <v>403</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F11" s="3">
         <v>138</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H11" s="10">
         <v>9150000</v>
@@ -1199,7 +1192,7 @@
         <v>1098000</v>
       </c>
       <c r="L11" s="6">
-        <f>+K11/12</f>
+        <f t="shared" si="5"/>
         <v>91500</v>
       </c>
       <c r="M11" s="9">
@@ -1207,9 +1200,9 @@
         <v>7594500</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="45.75">
+    <row r="12" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B12" s="13">
         <v>5</v>
@@ -1219,7 +1212,7 @@
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="4" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F12" s="3">
         <f>110.5+102.5</f>
@@ -1242,7 +1235,7 @@
         <v>1800000</v>
       </c>
       <c r="L12" s="6">
-        <f>+K12/12</f>
+        <f t="shared" si="5"/>
         <v>150000</v>
       </c>
       <c r="M12" s="9">
@@ -1250,9 +1243,9 @@
         <v>9600000</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="45.75">
+    <row r="13" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B13" s="13">
         <v>5</v>
@@ -1262,7 +1255,7 @@
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F13" s="3">
         <f>110.5+102.5</f>
@@ -1285,7 +1278,7 @@
         <v>1725000</v>
       </c>
       <c r="L13" s="6">
-        <f>+K13/12</f>
+        <f t="shared" si="5"/>
         <v>143750</v>
       </c>
       <c r="M13" s="9">
@@ -1293,9 +1286,9 @@
         <v>9200000</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="49.5" customHeight="1">
+    <row r="14" spans="1:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B14" s="13">
         <v>5</v>
@@ -1305,7 +1298,7 @@
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F14" s="3">
         <f>138+121.5</f>
@@ -1328,7 +1321,7 @@
         <v>1875000</v>
       </c>
       <c r="L14" s="6">
-        <f>+K14/12</f>
+        <f t="shared" si="5"/>
         <v>156250</v>
       </c>
       <c r="M14" s="9">
@@ -1336,30 +1329,32 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="I16" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="1">
-    <mergeCell ref="B1:M1"/>
-  </mergeCells>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="A3:A14">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="BLOQUEADO">
-      <formula>NOT(ISERROR(SEARCH("BLOQUEADO",A3)))</formula>
+    <cfRule type="beginsWith" dxfId="2" priority="1" operator="beginsWith" text="NO DISPONIBLE">
+      <formula>LEFT(A3,LEN("NO DISPONIBLE"))="NO DISPONIBLE"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A14">
     <cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="DISPONIBLE">
       <formula>LEFT(A3,LEN("DISPONIBLE"))="DISPONIBLE"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A14">
-    <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="NO DISPONIBLE">
-      <formula>LEFT(A3,LEN("NO DISPONIBLE"))="NO DISPONIBLE"</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="BLOQUEADO">
+      <formula>NOT(ISERROR(SEARCH("BLOQUEADO",A3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="7" scale="29" fitToWidth="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{833EE889-164E-4737-B5AC-37E94612D0EB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>